<commit_message>
feat(produzione-economica): listino PER ATTIVITÀ + "Scopri attività" + fix voce
Il DUNNING/DB hanno molte attività oltre alle 4 voci KPI. Il prezzo ora si aggancia all'ATTIVITÀ
(non più solo alla voce), così tutto il prodotto è valorizzabile.

- Migrazione additiva: acea_listino keyed per attività (voce/kpi restano come raggruppamento opzionale).
- Logica pura (TDD): normalizzaAttivita (chiave+etichetta); valorizza per attività; aggregaProduzione +perAttivita;
  fix voceDaAttivita (Revoca ≠ EL; "Rim Mis" → ERC).
- load.ts: prezzo per attività; SAL valorizzato per attività (via DB/master).
- Endpoint: CRUD listino per attività + POST /listino/scopri (popola il listino dalle attività reali a €0).
- UI: editor per attività con "Scopri attività dai dati"; tabella "Produzione per attività".
- Export Excel: blocco Attività nel template + fallback.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/Produzione-Economica-Dashboard.xlsx
+++ b/public/templates/Produzione-Economica-Dashboard.xlsx
@@ -931,13 +931,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J32"/>
+  <dimension ref="A1:N41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="32" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -981,6 +983,21 @@
           <t>Produzione</t>
         </is>
       </c>
+      <c r="L1" s="6" t="inlineStr">
+        <is>
+          <t>Attività</t>
+        </is>
+      </c>
+      <c r="M1" s="6" t="inlineStr">
+        <is>
+          <t>Ordini</t>
+        </is>
+      </c>
+      <c r="N1" s="6" t="inlineStr">
+        <is>
+          <t>Produzione</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr"/>
@@ -1001,6 +1018,13 @@
       <c r="J2" s="8" t="n">
         <v>0</v>
       </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" s="8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr"/>
@@ -1021,6 +1045,13 @@
       <c r="J3" s="8" t="n">
         <v>0</v>
       </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" s="8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr"/>
@@ -1041,6 +1072,13 @@
       <c r="J4" s="8" t="n">
         <v>0</v>
       </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" s="8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr"/>
@@ -1061,6 +1099,13 @@
       <c r="J5" s="8" t="n">
         <v>0</v>
       </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" s="8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr"/>
@@ -1081,6 +1126,13 @@
       <c r="J6" s="8" t="n">
         <v>0</v>
       </c>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" s="8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr"/>
@@ -1101,6 +1153,13 @@
       <c r="J7" s="8" t="n">
         <v>0</v>
       </c>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" s="8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr"/>
@@ -1121,6 +1180,13 @@
       <c r="J8" s="8" t="n">
         <v>0</v>
       </c>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" s="8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr"/>
@@ -1141,6 +1207,13 @@
       <c r="J9" s="8" t="n">
         <v>0</v>
       </c>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" s="8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr"/>
@@ -1161,6 +1234,13 @@
       <c r="J10" s="8" t="n">
         <v>0</v>
       </c>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="n">
+        <v>0</v>
+      </c>
+      <c r="N10" s="8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr"/>
@@ -1181,6 +1261,13 @@
       <c r="J11" s="8" t="n">
         <v>0</v>
       </c>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" s="8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr"/>
@@ -1201,6 +1288,13 @@
       <c r="J12" s="8" t="n">
         <v>0</v>
       </c>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" s="8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr"/>
@@ -1221,6 +1315,13 @@
       <c r="J13" s="8" t="n">
         <v>0</v>
       </c>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" s="8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr"/>
@@ -1241,6 +1342,13 @@
       <c r="J14" s="8" t="n">
         <v>0</v>
       </c>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" s="8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr"/>
@@ -1261,6 +1369,13 @@
       <c r="J15" s="8" t="n">
         <v>0</v>
       </c>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" s="8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr"/>
@@ -1281,100 +1396,300 @@
       <c r="J16" s="8" t="n">
         <v>0</v>
       </c>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" s="8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="I17" t="inlineStr"/>
       <c r="J17" s="8" t="n">
         <v>0</v>
       </c>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="n">
+        <v>0</v>
+      </c>
+      <c r="N17" s="8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="I18" t="inlineStr"/>
       <c r="J18" s="8" t="n">
         <v>0</v>
       </c>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="n">
+        <v>0</v>
+      </c>
+      <c r="N18" s="8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="19">
       <c r="I19" t="inlineStr"/>
       <c r="J19" s="8" t="n">
         <v>0</v>
       </c>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N19" s="8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="I20" t="inlineStr"/>
       <c r="J20" s="8" t="n">
         <v>0</v>
       </c>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="n">
+        <v>0</v>
+      </c>
+      <c r="N20" s="8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="I21" t="inlineStr"/>
       <c r="J21" s="8" t="n">
         <v>0</v>
       </c>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="n">
+        <v>0</v>
+      </c>
+      <c r="N21" s="8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="22">
       <c r="I22" t="inlineStr"/>
       <c r="J22" s="8" t="n">
         <v>0</v>
       </c>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="n">
+        <v>0</v>
+      </c>
+      <c r="N22" s="8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="I23" t="inlineStr"/>
       <c r="J23" s="8" t="n">
         <v>0</v>
       </c>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="n">
+        <v>0</v>
+      </c>
+      <c r="N23" s="8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="24">
       <c r="I24" t="inlineStr"/>
       <c r="J24" s="8" t="n">
         <v>0</v>
       </c>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="n">
+        <v>0</v>
+      </c>
+      <c r="N24" s="8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="25">
       <c r="I25" t="inlineStr"/>
       <c r="J25" s="8" t="n">
         <v>0</v>
       </c>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="n">
+        <v>0</v>
+      </c>
+      <c r="N25" s="8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="26">
       <c r="I26" t="inlineStr"/>
       <c r="J26" s="8" t="n">
         <v>0</v>
       </c>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="n">
+        <v>0</v>
+      </c>
+      <c r="N26" s="8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="27">
       <c r="I27" t="inlineStr"/>
       <c r="J27" s="8" t="n">
         <v>0</v>
       </c>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="n">
+        <v>0</v>
+      </c>
+      <c r="N27" s="8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="28">
       <c r="I28" t="inlineStr"/>
       <c r="J28" s="8" t="n">
         <v>0</v>
       </c>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="n">
+        <v>0</v>
+      </c>
+      <c r="N28" s="8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="29">
       <c r="I29" t="inlineStr"/>
       <c r="J29" s="8" t="n">
         <v>0</v>
       </c>
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="n">
+        <v>0</v>
+      </c>
+      <c r="N29" s="8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="30">
       <c r="I30" t="inlineStr"/>
       <c r="J30" s="8" t="n">
         <v>0</v>
       </c>
+      <c r="L30" t="inlineStr"/>
+      <c r="M30" t="n">
+        <v>0</v>
+      </c>
+      <c r="N30" s="8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="31">
       <c r="I31" t="inlineStr"/>
       <c r="J31" s="8" t="n">
         <v>0</v>
       </c>
+      <c r="L31" t="inlineStr"/>
+      <c r="M31" t="n">
+        <v>0</v>
+      </c>
+      <c r="N31" s="8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="32">
       <c r="I32" t="inlineStr"/>
       <c r="J32" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L32" t="inlineStr"/>
+      <c r="M32" t="n">
+        <v>0</v>
+      </c>
+      <c r="N32" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="L33" t="inlineStr"/>
+      <c r="M33" t="n">
+        <v>0</v>
+      </c>
+      <c r="N33" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="L34" t="inlineStr"/>
+      <c r="M34" t="n">
+        <v>0</v>
+      </c>
+      <c r="N34" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="L35" t="inlineStr"/>
+      <c r="M35" t="n">
+        <v>0</v>
+      </c>
+      <c r="N35" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="L36" t="inlineStr"/>
+      <c r="M36" t="n">
+        <v>0</v>
+      </c>
+      <c r="N36" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="L37" t="inlineStr"/>
+      <c r="M37" t="n">
+        <v>0</v>
+      </c>
+      <c r="N37" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="L38" t="inlineStr"/>
+      <c r="M38" t="n">
+        <v>0</v>
+      </c>
+      <c r="N38" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="L39" t="inlineStr"/>
+      <c r="M39" t="n">
+        <v>0</v>
+      </c>
+      <c r="N39" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="L40" t="inlineStr"/>
+      <c r="M40" t="n">
+        <v>0</v>
+      </c>
+      <c r="N40" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="L41" t="inlineStr"/>
+      <c r="M41" t="n">
+        <v>0</v>
+      </c>
+      <c r="N41" s="8" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>